<commit_message>
R-Auswertung erweitert + .gitignore aufgeräumt
- R/laufzeiten-auswerten.R: weitere Auswertungs-Tabellen (Top-Themen,
  Sachgebiete-Zeitreihe, Parteien-Index).
- .gitignore: R-Projekt-Files, docs/, texte/ ausgeschlossen.
- data/: aktualisierte Auswertungs-XLSX inkl. neuer ALLE_topthemen_zeitreihe
  und index_parteien.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ALLE_sachgebiete_zeitreihe.xlsx
+++ b/data/ALLE_sachgebiete_zeitreihe.xlsx
@@ -10838,13 +10838,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0E4B0439-E797-4267-A306-E8CCE7A53BD3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0F7B2248-DF70-44E7-9CAA-5D973AD790D8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D649E2CB-CB5B-431A-B693-3C920300C14A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FB8A0491-0A7F-4B8E-9961-4963B545F110}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B28CA16-6B0C-45A1-8971-E0B5F4B23BCA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07B682FF-0C56-4988-89CF-AFC954459DDB}"/>
 </file>
</xml_diff>